<commit_message>
Added the explanatory document for problem 2nd
</commit_message>
<xml_diff>
--- a/Problem C/Problem 1st/result/result1-release.xlsx
+++ b/Problem C/Problem 1st/result/result1-release.xlsx
@@ -5,14 +5,16 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\My\2026CUMCM-share\Problem C\Problem 1st\Problem 1st\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\My\2026CUMCM-share\Problem C\Problem 1st\result\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="10571" windowHeight="9024"/>
+    <workbookView windowWidth="10680" windowHeight="9024" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="表1" sheetId="3" r:id="rId2"/>
+    <sheet name="表2" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="166">
   <si>
     <t>时间段</t>
   </si>
@@ -476,6 +478,60 @@
   </si>
   <si>
     <t>0:00+1-0:10+1</t>
+  </si>
+  <si>
+    <t>10：00-10：10</t>
+  </si>
+  <si>
+    <t>12：00-12：10</t>
+  </si>
+  <si>
+    <t>14：00-14：10</t>
+  </si>
+  <si>
+    <t>16：00-16：10</t>
+  </si>
+  <si>
+    <t>18：00-18：10</t>
+  </si>
+  <si>
+    <t>20：00-20：10</t>
+  </si>
+  <si>
+    <t>全天购电量</t>
+  </si>
+  <si>
+    <t>全天购电费</t>
+  </si>
+  <si>
+    <t>充电量</t>
+  </si>
+  <si>
+    <t>放电量</t>
+  </si>
+  <si>
+    <t>0:00-4:00</t>
+  </si>
+  <si>
+    <t>12:00-16:00</t>
+  </si>
+  <si>
+    <t>4:00-8:00</t>
+  </si>
+  <si>
+    <t>16:00-20:00</t>
+  </si>
+  <si>
+    <t>8:00-12:00</t>
+  </si>
+  <si>
+    <t>20:00-24:00</t>
+  </si>
+  <si>
+    <t>0：00储电量</t>
+  </si>
+  <si>
+    <t>24：00储电量</t>
   </si>
 </sst>
 </file>
@@ -488,7 +544,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -497,8 +553,14 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -951,153 +1013,160 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1447,7 +1516,8 @@
   <dimension ref="A1:D145"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="3"/>
   <cols>
-    <col min="2" max="2" width="9.66666666666667"/>
+    <col min="1" max="1" width="17.7777777777778" customWidth="1"/>
+    <col min="2" max="2" width="10.6666666666667"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -3484,4 +3554,229 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="5"/>
+  <cols>
+    <col min="1" max="1" width="20.7777777777778" customWidth="1"/>
+    <col min="2" max="2" width="10.6666666666667"/>
+    <col min="3" max="3" width="19.5555555555556" customWidth="1"/>
+    <col min="4" max="4" width="10.6666666666667"/>
+    <col min="5" max="5" width="25.5555555555556" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>149</v>
+      </c>
+      <c r="D2">
+        <v>486.4029</v>
+      </c>
+      <c r="E2" t="s">
+        <v>150</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" t="s">
+        <v>151</v>
+      </c>
+      <c r="B3">
+        <v>394.93148</v>
+      </c>
+      <c r="C3" t="s">
+        <v>152</v>
+      </c>
+      <c r="D3">
+        <v>636.98262</v>
+      </c>
+      <c r="E3" t="s">
+        <v>153</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4">
+        <v>59482.7</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="E4" s="3"/>
+      <c r="F4">
+        <v>35126.95</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="6" outlineLevelCol="5"/>
+  <cols>
+    <col min="2" max="2" width="10.6666666666667"/>
+    <col min="3" max="3" width="9.66666666666667"/>
+    <col min="5" max="6" width="10.6666666666667"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="B2" s="2">
+        <v>4500</v>
+      </c>
+      <c r="C2" s="2">
+        <v>0</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="E2" s="2">
+        <v>5286.0352</v>
+      </c>
+      <c r="F2" s="2">
+        <v>91.1014</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="B3" s="2">
+        <v>833.3333</v>
+      </c>
+      <c r="C3" s="2">
+        <v>6365.8412</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="E3" s="2">
+        <v>0</v>
+      </c>
+      <c r="F3" s="2">
+        <v>5780.1319</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B4" s="2">
+        <v>4787.9643</v>
+      </c>
+      <c r="C4" s="2">
+        <v>1702.997</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="E4" s="2">
+        <v>5333.3333</v>
+      </c>
+      <c r="F4" s="2">
+        <v>2859.8681</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5">
+        <v>6000</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="E5" s="1"/>
+      <c r="F5">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="D5:E5"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>